<commit_message>
docs: add Phase 7 test execution reports, Excel workbooks, HTML dashboards, and load testing artifacts
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -41,8 +41,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B71C1C"/>
-        <bgColor rgb="00B71C1C"/>
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +65,7 @@
         <color rgb="00D9D9D9"/>
       </top>
       <bottom style="medium">
-        <color rgb="00B71C1C"/>
+        <color rgb="001F497D"/>
       </bottom>
     </border>
   </borders>
@@ -442,15 +442,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -466,20 +465,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Test Name</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Execution Time (s)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Execution Time (s)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>

</xml_diff>

<commit_message>
docs: add Android Appium E2E reports, Excel workbooks, GitHub Pages artifacts, and summary
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -41,8 +41,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F497D"/>
-        <bgColor rgb="001F497D"/>
+        <fgColor rgb="00B71C1C"/>
+        <bgColor rgb="00B71C1C"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +65,7 @@
         <color rgb="00D9D9D9"/>
       </top>
       <bottom style="medium">
-        <color rgb="001F497D"/>
+        <color rgb="00B71C1C"/>
       </bottom>
     </border>
   </borders>
@@ -442,14 +442,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -465,15 +466,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Execution Time (s)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>

</xml_diff>